<commit_message>
第2轮评测 - compare cleaned.json --type weekly --date 2026-06。
</commit_message>
<xml_diff>
--- a/test/output/report.xlsx
+++ b/test/output/report.xlsx
@@ -419,7 +419,7 @@
         <v>总销售额</v>
       </c>
       <c r="B2">
-        <v>1299</v>
+        <v>11298</v>
       </c>
     </row>
     <row r="3">
@@ -427,7 +427,7 @@
         <v>订单数</v>
       </c>
       <c r="B3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -435,7 +435,7 @@
         <v>总销量</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5">
@@ -451,7 +451,7 @@
         <v>日均销售额</v>
       </c>
       <c r="B6">
-        <v>1299</v>
+        <v>11298</v>
       </c>
     </row>
     <row r="7">
@@ -459,7 +459,7 @@
         <v>客单价</v>
       </c>
       <c r="B7">
-        <v>1299</v>
+        <v>5649</v>
       </c>
     </row>
     <row r="8">
@@ -467,7 +467,7 @@
         <v>单笔最高</v>
       </c>
       <c r="B8">
-        <v>1299</v>
+        <v>9999</v>
       </c>
     </row>
     <row r="9">
@@ -483,7 +483,7 @@
         <v>活跃渠道数</v>
       </c>
       <c r="B10">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -529,13 +529,13 @@
         <v>星期一</v>
       </c>
       <c r="C2">
-        <v>1299</v>
+        <v>11298</v>
       </c>
       <c r="D2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <cols>
     <col min="1" max="1" width="8.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -582,31 +582,51 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
+        <v>新渠道</v>
+      </c>
+      <c r="C2">
+        <v>9999</v>
+      </c>
+      <c r="D2">
+        <v>0.8850238980350504</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
         <v>未分类</v>
       </c>
-      <c r="C2">
+      <c r="C3">
         <v>1299</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2">
+      <c r="D3">
+        <v>0.11497610196494955</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D54"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1322,9 +1342,51 @@
         <v>1</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-03-03</v>
+      </c>
+      <c r="B52">
+        <v>1599</v>
+      </c>
+      <c r="C52" t="str">
+        <v>淘宝</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-05-01</v>
+      </c>
+      <c r="B53">
+        <v>1999</v>
+      </c>
+      <c r="C53" t="str">
+        <v>抖音</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-06-08</v>
+      </c>
+      <c r="B54">
+        <v>9999</v>
+      </c>
+      <c r="C54" t="str">
+        <v>新渠道</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D54"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
第3轮评测 - clean imported.json 处理 2026-02-31、2026-04-31 这类日期。
</commit_message>
<xml_diff>
--- a/test/output/report.xlsx
+++ b/test/output/report.xlsx
@@ -626,7 +626,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D52"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1344,49 +1344,21 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>2026-03-03</v>
+        <v>2026-06-08</v>
       </c>
       <c r="B52">
-        <v>1599</v>
+        <v>9999</v>
       </c>
       <c r="C52" t="str">
-        <v>淘宝</v>
+        <v>新渠道</v>
       </c>
       <c r="D52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>2026-05-01</v>
-      </c>
-      <c r="B53">
-        <v>1999</v>
-      </c>
-      <c r="C53" t="str">
-        <v>抖音</v>
-      </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>2026-06-08</v>
-      </c>
-      <c r="B54">
-        <v>9999</v>
-      </c>
-      <c r="C54" t="str">
-        <v>新渠道</v>
-      </c>
-      <c r="D54">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D54"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D52"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>